<commit_message>
Update Synthetic Data.xlsx for Week 1 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="4" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name=" Dict 1" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="240">
   <si>
     <t>signup_date</t>
   </si>
@@ -759,6 +759,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -791,7 +795,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -816,6 +820,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -826,11 +842,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -870,14 +887,44 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -1376,9 +1423,319 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45872</v>
+      </c>
+      <c r="D2" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>45903</v>
+      </c>
+      <c r="D3" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="G3">
+        <f>Loan!D28</f>
+        <v>27133.333333333332</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3">
+        <v>45933</v>
+      </c>
+      <c r="D4" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
+        <v>45903</v>
+      </c>
+      <c r="D5" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="2">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3">
+        <v>45933</v>
+      </c>
+      <c r="D6" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3">
+        <v>45964</v>
+      </c>
+      <c r="D7" s="10" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="28">
+        <v>1</v>
+      </c>
+      <c r="C8" s="29">
+        <v>45874</v>
+      </c>
+      <c r="D8" s="30" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="28">
+        <v>2</v>
+      </c>
+      <c r="C9" s="29">
+        <v>45905</v>
+      </c>
+      <c r="D9" s="30" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="28">
+        <v>3</v>
+      </c>
+      <c r="C10" s="29">
+        <v>45935</v>
+      </c>
+      <c r="D10" s="31" t="e">
+        <f>D9</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="13">
+        <v>45937</v>
+      </c>
+      <c r="D11" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="2">
+        <v>2</v>
+      </c>
+      <c r="C12" s="13">
+        <v>45968</v>
+      </c>
+      <c r="D12" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2">
+        <v>3</v>
+      </c>
+      <c r="C13" s="13">
+        <v>45998</v>
+      </c>
+      <c r="D13" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="2">
+        <v>2</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="2">
+        <v>3</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6" t="e">
+        <f>#REF!/#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2753,17 +3110,17 @@
     <col min="2" max="2" width="11.26953125" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" style="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.36328125" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" style="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" style="26" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.36328125" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.36328125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>57</v>
       </c>
@@ -2776,7 +3133,7 @@
       <c r="D1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="21" t="s">
         <v>29</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -2785,10 +3142,10 @@
       <c r="G1" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="25" t="s">
         <v>97</v>
       </c>
       <c r="J1" s="5" t="s">
@@ -2814,7 +3171,7 @@
       <c r="D2" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="22">
         <v>300000</v>
       </c>
       <c r="F2" s="7">
@@ -2823,10 +3180,10 @@
       <c r="G2" s="7">
         <v>725</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="24">
         <v>20000</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="24">
         <v>29500</v>
       </c>
       <c r="J2" s="7" t="s">
@@ -2852,7 +3209,7 @@
       <c r="D3" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="22">
         <v>100000</v>
       </c>
       <c r="F3" s="7">
@@ -2861,10 +3218,10 @@
       <c r="G3" s="7">
         <v>650</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="24">
         <v>15000</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="24">
         <v>18500</v>
       </c>
       <c r="J3" s="7" t="s">
@@ -2890,7 +3247,7 @@
       <c r="D4" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="22">
         <v>500000</v>
       </c>
       <c r="F4" s="7">
@@ -2899,10 +3256,10 @@
       <c r="G4" s="7">
         <v>780</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="24">
         <v>30000</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="24">
         <v>37000</v>
       </c>
       <c r="J4" s="7" t="s">
@@ -2928,7 +3285,7 @@
       <c r="D5" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="22">
         <v>600000</v>
       </c>
       <c r="F5" s="7">
@@ -2937,10 +3294,10 @@
       <c r="G5" s="7">
         <v>590</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="24">
         <v>45000</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="24">
         <v>43000</v>
       </c>
       <c r="J5" s="7" t="s">
@@ -2966,7 +3323,7 @@
       <c r="D6" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="22">
         <v>80000</v>
       </c>
       <c r="F6" s="7">
@@ -2975,10 +3332,10 @@
       <c r="G6" s="7">
         <v>520</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="24">
         <v>22000</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="24">
         <v>28500</v>
       </c>
       <c r="J6" s="7" t="s">
@@ -3004,7 +3361,7 @@
       <c r="D7" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="22">
         <v>700000</v>
       </c>
       <c r="F7" s="7">
@@ -3013,10 +3370,10 @@
       <c r="G7" s="7">
         <v>735</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="24">
         <v>35000</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="24">
         <v>47000</v>
       </c>
       <c r="J7" s="7" t="s">
@@ -3042,7 +3399,7 @@
       <c r="D8" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="22">
         <v>200000</v>
       </c>
       <c r="F8" s="7">
@@ -3051,10 +3408,10 @@
       <c r="G8" s="7">
         <v>680</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="24">
         <v>12000</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="24">
         <v>21000</v>
       </c>
       <c r="J8" s="7" t="s">
@@ -3080,7 +3437,7 @@
       <c r="D9" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="22">
         <v>1000000</v>
       </c>
       <c r="F9" s="7">
@@ -3089,10 +3446,10 @@
       <c r="G9" s="7">
         <v>760</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="24">
         <v>60000</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="24">
         <v>52000</v>
       </c>
       <c r="J9" s="7" t="s">
@@ -3118,7 +3475,7 @@
       <c r="D10" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="22">
         <v>120000</v>
       </c>
       <c r="F10" s="7">
@@ -3127,10 +3484,10 @@
       <c r="G10" s="7">
         <v>605</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="24">
         <v>18000</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="24">
         <v>21000</v>
       </c>
       <c r="J10" s="7" t="s">
@@ -3156,7 +3513,7 @@
       <c r="D11" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="22">
         <v>350000</v>
       </c>
       <c r="F11" s="7">
@@ -3165,10 +3522,10 @@
       <c r="G11" s="7">
         <v>745</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="24">
         <v>20000</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="24">
         <v>33000</v>
       </c>
       <c r="J11" s="7" t="s">
@@ -3194,7 +3551,7 @@
       <c r="D12" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="22">
         <v>120000</v>
       </c>
       <c r="F12" s="7">
@@ -3203,10 +3560,10 @@
       <c r="G12" s="7">
         <v>730</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="24">
         <v>15000</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="24">
         <v>22000</v>
       </c>
       <c r="J12" s="7" t="s">
@@ -3232,7 +3589,7 @@
       <c r="D13" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="22">
         <v>900000</v>
       </c>
       <c r="F13" s="7">
@@ -3241,10 +3598,10 @@
       <c r="G13" s="7">
         <v>790</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="24">
         <v>40000</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="24">
         <v>61000</v>
       </c>
       <c r="J13" s="7" t="s">
@@ -3270,7 +3627,7 @@
       <c r="D14" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="22">
         <v>250000</v>
       </c>
       <c r="F14" s="7">
@@ -3279,10 +3636,10 @@
       <c r="G14" s="7">
         <v>540</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="24">
         <v>25000</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="24">
         <v>26000</v>
       </c>
       <c r="J14" s="7" t="s">
@@ -3308,7 +3665,7 @@
       <c r="D15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="22">
         <v>150000</v>
       </c>
       <c r="F15" s="7">
@@ -3317,10 +3674,10 @@
       <c r="G15" s="7">
         <v>770</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="24">
         <v>18000</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="24">
         <v>24000</v>
       </c>
       <c r="J15" s="7" t="s">
@@ -3346,7 +3703,7 @@
       <c r="D16" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="22">
         <v>300000</v>
       </c>
       <c r="F16" s="7">
@@ -3355,10 +3712,10 @@
       <c r="G16" s="7">
         <v>610</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="24">
         <v>28000</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="24">
         <v>31000</v>
       </c>
       <c r="J16" s="7" t="s">
@@ -3554,7 +3911,7 @@
       <c r="I4" s="8">
         <v>46300</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="17" t="s">
         <v>225</v>
       </c>
       <c r="K4" s="7">
@@ -4196,7 +4553,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="18" t="s">
         <v>238</v>
       </c>
     </row>
@@ -4250,16 +4607,13 @@
         <f>K2/H2</f>
         <v>19000</v>
       </c>
-      <c r="F25" t="s">
-        <v>66</v>
-      </c>
       <c r="G25" s="13"/>
       <c r="H25" s="16">
-        <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
+        <f>SUMIFS(D25:D27, A25:A27,A2, C25:C27, "&lt;="&amp;C27)</f>
         <v>57000</v>
       </c>
       <c r="I25" s="6">
-        <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
+        <f>SUMIFS(D25:D27, A25:A27,A2, C25:C27, "&lt;="&amp;C27)</f>
         <v>57000</v>
       </c>
       <c r="J25" s="20" t="s">
@@ -4319,7 +4673,7 @@
         <f>SUMIFS(D28:D30, A28:A30,A3,C28:C30,"&lt;="&amp;C30)</f>
         <v>81400</v>
       </c>
-      <c r="J28" s="18" t="s">
+      <c r="J28" s="19" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4354,46 +4708,46 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="28">
         <v>1</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="29">
         <v>45874</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="30">
         <f>K4/H4</f>
         <v>32666.666666666668</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="28">
         <v>2</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="29">
         <v>45905</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="30">
         <f>K4/H4</f>
         <v>32666.666666666668</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="28">
         <v>3</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="29">
         <v>45935</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="31">
         <f>D32</f>
         <v>32666.666666666668</v>
       </c>
@@ -4405,7 +4759,7 @@
         <f>SUMIFS(D31:D32,A31:A32, A4,C31:C32, "&lt;="&amp;C33)</f>
         <v>65333.333333333336</v>
       </c>
-      <c r="J33" s="19">
+      <c r="J33" s="27">
         <f>MAX(0,H33-I33)</f>
         <v>32666.666666666664</v>
       </c>

</xml_diff>

<commit_message>
Update Synthetic Data and Input Data for Week 2 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="3" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="3" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Datagrain" sheetId="3" r:id="rId1"/>
@@ -997,12 +997,21 @@
   </cellStyles>
   <dxfs count="13">
     <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1024,21 +1033,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
@@ -1126,19 +1126,19 @@
     <tableColumn id="4" name="amount_due" dataDxfId="9" dataCellStyle="Comma"/>
     <tableColumn id="5" name="payment_date" dataDxfId="8"/>
     <tableColumn id="6" name="Scenario"/>
-    <tableColumn id="7" name="Payment_amount" dataDxfId="6" dataCellStyle="Comma"/>
-    <tableColumn id="8" name="outstanding" dataDxfId="5" dataCellStyle="Comma"/>
-    <tableColumn id="9" name="cumulative_due" dataDxfId="2" dataCellStyle="Comma"/>
-    <tableColumn id="10" name="cumulative_paid" dataDxfId="0" dataCellStyle="Comma"/>
-    <tableColumn id="11" name="cumulative_arrears_amount" dataDxfId="1" dataCellStyle="Comma"/>
-    <tableColumn id="12" name="Oldest Unpaid Due Date" dataDxfId="4"/>
-    <tableColumn id="13" name="DPD" dataDxfId="7">
+    <tableColumn id="7" name="Payment_amount" dataDxfId="7" dataCellStyle="Comma"/>
+    <tableColumn id="8" name="outstanding" dataDxfId="6" dataCellStyle="Comma"/>
+    <tableColumn id="9" name="cumulative_due" dataDxfId="5" dataCellStyle="Comma"/>
+    <tableColumn id="10" name="cumulative_paid" dataDxfId="4" dataCellStyle="Comma"/>
+    <tableColumn id="11" name="cumulative_arrears_amount" dataDxfId="3" dataCellStyle="Comma"/>
+    <tableColumn id="12" name="Oldest Unpaid Due Date" dataDxfId="2"/>
+    <tableColumn id="13" name="DPD" dataDxfId="1">
       <calculatedColumnFormula>MAX(0,L43-Table1[[#This Row],[due_date]])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="14" name="Bucket">
       <calculatedColumnFormula>IF(M2="","Current",IF(M2&lt;=0,"Current",IF(M2&lt;=7,"1–7",IF(M2&lt;=30,"8–30",IF(M2&lt;=60,"31–60",IF(M2&lt;=90,"61–90","90+"))))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" name="reporting_date " dataDxfId="3">
+    <tableColumn id="15" name="reporting_date " dataDxfId="0">
       <calculatedColumnFormula>L62</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5353,7 +5353,7 @@
         <v>14000</v>
       </c>
       <c r="H10" s="13">
-        <f t="shared" ref="H9:H10" si="4">D10-G10</f>
+        <f t="shared" ref="H10" si="4">D10-G10</f>
         <v>18666.666666666668</v>
       </c>
       <c r="I10" s="13">
@@ -6054,7 +6054,7 @@
         <v>90+</v>
       </c>
       <c r="O23" s="18">
-        <v>45990</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update Input Data for Week 2 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -9,17 +9,21 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="4" r:id="rId1"/>
-    <sheet name="Metric" sheetId="14" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="15" r:id="rId3"/>
-    <sheet name="Application" sheetId="5" r:id="rId4"/>
-    <sheet name="Loan" sheetId="2" r:id="rId5"/>
-    <sheet name="Installment" sheetId="12" r:id="rId6"/>
-    <sheet name="Formula Allocation" sheetId="13" r:id="rId7"/>
+    <sheet name="Application" sheetId="5" r:id="rId2"/>
+    <sheet name="Loan" sheetId="2" r:id="rId3"/>
+    <sheet name="Installment" sheetId="12" r:id="rId4"/>
+    <sheet name="Formula Allocation" sheetId="13" r:id="rId5"/>
+    <sheet name="Metric" sheetId="14" r:id="rId6"/>
+    <sheet name="Reconcilation" sheetId="15" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="16" r:id="rId8"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId9"/>
+  </externalReferences>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="282">
   <si>
     <t>signup_date</t>
   </si>
@@ -762,17 +766,134 @@
   </si>
   <si>
     <t>Total principal disbursed</t>
+  </si>
+  <si>
+    <t>Total contract value — flat formula (₦)</t>
+  </si>
+  <si>
+    <t>Sum of all instalment amount_due (₦)</t>
+  </si>
+  <si>
+    <t>Loan Repayment Dashboard</t>
+  </si>
+  <si>
+    <t>Nigerian microfinance loan book — disbursements, collections &amp; delinquency</t>
+  </si>
+  <si>
+    <t>Controls</t>
+  </si>
+  <si>
+    <t>Channel filter: source data does not currently capture acquisition_channel at customer level (see Reconciliation tab) — filter is provided for future use and defaults to 'All'.</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Portfolio Snapshot</t>
+  </si>
+  <si>
+    <t>Delinquency by DPD Bucket</t>
+  </si>
+  <si>
+    <t>Loan Count (units)</t>
+  </si>
+  <si>
+    <t>% of Loans</t>
+  </si>
+  <si>
+    <t>Arrears Value (₦)</t>
+  </si>
+  <si>
+    <t>Outstanding Principal at Risk (₦)</t>
+  </si>
+  <si>
+    <t>% of Outstanding Principal</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>1-7</t>
+  </si>
+  <si>
+    <t>8-30</t>
+  </si>
+  <si>
+    <t>31-60</t>
+  </si>
+  <si>
+    <t>61-90</t>
+  </si>
+  <si>
+    <t>90+</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Exposure by Product &amp; Origination Month</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>Values = principal disbursed (₦), filtered by Reporting Date, Product, Channel and Customer Type above.</t>
+  </si>
+  <si>
+    <t>Actions Supported by These Results</t>
+  </si>
+  <si>
+    <t>1. Trigger early collections outreach at first delinquency (1–7 DPD), not just at 90+.</t>
+  </si>
+  <si>
+    <t>Every currently delinquent loan in the book has already crossed 90+ DPD — there is currently no population sitting in the 1–60 day buckets. That means the book's early-warning stage is effectively empty: loans appear to jump straight from Current to severely delinquent, most likely because collections only start once accounts are already very late. Add a structured outreach step (SMS/call) as soon as an instalment is 1–7 days overdue.</t>
+  </si>
+  <si>
+    <t>Owner:</t>
+  </si>
+  <si>
+    <t>Collections Team Lead</t>
+  </si>
+  <si>
+    <t>Monitoring metric:</t>
+  </si>
+  <si>
+    <t>Loan count and ₦ value in the 1–7, 8–30 and 31–60 DPD buckets (Dashboard delinquency table) — review weekly. If this population stays near zero after the process is live, it confirms loans are genuinely cured quickly; if it starts filling and 90+ volume falls, it shows the new step is catching cases before they become severely delinquent.</t>
+  </si>
+  <si>
+    <t>2. Reconcile the 3 loans with missing payment-amount data before reporting collection rate externally.</t>
+  </si>
+  <si>
+    <t>L015, L016 and L018 (₦435,600 of contractual exposure, ~15% of the book) have a payment_date recorded but no payment_amount in the source system, so this dashboard conservatively treats them as ₦0 collected. If payments were in fact received, both Amount Collected and Collection Rate are currently understated, and these three loans are overstated in the 90+ bucket.</t>
+  </si>
+  <si>
+    <t>Data/Systems Analyst (Loan Operations), with sign-off from Finance before external reporting</t>
+  </si>
+  <si>
+    <t>Count of Installment rows with a payment_date but blank payment_amount (Reconciliation tab, issue log row 4) — target zero before each external report; re-check portfolio Collection Rate once fixed.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="167" formatCode="\₦#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -828,8 +949,69 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -846,6 +1028,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDE7"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFDE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -878,7 +1090,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -978,6 +1190,62 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="167" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1104,6 +1372,1773 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Loan Count by DPD Bucket (units) — as of Reporting Date (cell C6 above)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>[1]Dashboard!$C$19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Loan Count (units)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4F81BD"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>[1]Dashboard!$B$20:$B$25</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Current</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1-7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8-30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31-60</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>61-90</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>90+</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Dashboard!$C$20:$C$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="356125320"/>
+        <c:axId val="356125712"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="356125320"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>DPD bucket</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="356125712"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="356125712"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="B3B3B3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Number of loans (count)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="356125320"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Principal Disbursed by Product &amp; Origination Month (₦ Naira) — as of Reporting Date (cell C6 above)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>[1]Dashboard!$C$29</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Business Loan</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4F81BD"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>[1]Dashboard!$B$30:$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2025-07</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2025-08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025-09</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Dashboard!$C$30:$C$33</c:f>
+              <c:numCache>
+                <c:formatCode>\₦#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>530000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>110000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>[1]Dashboard!$D$29</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Personal Loan</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C0504D"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>[1]Dashboard!$B$30:$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2025-07</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2025-08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025-09</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Dashboard!$D$30:$D$33</c:f>
+              <c:numCache>
+                <c:formatCode>\₦#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>935000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>[1]Dashboard!$E$29</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Salary Advance</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="9BBB59"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>[1]Dashboard!$B$30:$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2025-07</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2025-08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2025-09</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Dashboard!$E$30:$E$33</c:f>
+              <c:numCache>
+                <c:formatCode>\₦#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>430000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>70000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>130000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="356127280"/>
+        <c:axId val="356128848"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="356127280"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Origination month</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="356128848"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="356128848"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="B3B3B3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Principal disbursed (₦ Naira)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="\₦#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="356127280"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>61880</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>111280</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>61880</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>111130</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Dashboard"/>
+      <sheetName val="Metric Definitions"/>
+      <sheetName val="Reconciliation"/>
+      <sheetName val="Data - Customer"/>
+      <sheetName val="Data - Application"/>
+      <sheetName val="Data - Loan"/>
+      <sheetName val="Data - Installment"/>
+      <sheetName val="Calc - Installment"/>
+      <sheetName val="Calc - Loan Summary"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="19">
+          <cell r="C19" t="str">
+            <v>Loan Count (units)</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="B20" t="str">
+            <v>Current</v>
+          </cell>
+          <cell r="C20">
+            <v>11</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="B21" t="str">
+            <v>1-7</v>
+          </cell>
+          <cell r="C21">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="B22" t="str">
+            <v>8-30</v>
+          </cell>
+          <cell r="C22">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="B23" t="str">
+            <v>31-60</v>
+          </cell>
+          <cell r="C23">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="B24" t="str">
+            <v>61-90</v>
+          </cell>
+          <cell r="C24">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="B25" t="str">
+            <v>90+</v>
+          </cell>
+          <cell r="C25">
+            <v>9</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="C29" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D29" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="E29" t="str">
+            <v>Salary Advance</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="B30" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="C30">
+            <v>530000</v>
+          </cell>
+          <cell r="D30">
+            <v>935000</v>
+          </cell>
+          <cell r="E30">
+            <v>430000</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="B31" t="str">
+            <v>2025-08</v>
+          </cell>
+          <cell r="C31">
+            <v>0</v>
+          </cell>
+          <cell r="D31">
+            <v>0</v>
+          </cell>
+          <cell r="E31">
+            <v>70000</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="B32" t="str">
+            <v>2025-09</v>
+          </cell>
+          <cell r="C32">
+            <v>110000</v>
+          </cell>
+          <cell r="D32">
+            <v>0</v>
+          </cell>
+          <cell r="E32">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="B33" t="str">
+            <v>2025-10</v>
+          </cell>
+          <cell r="C33">
+            <v>0</v>
+          </cell>
+          <cell r="D33">
+            <v>0</v>
+          </cell>
+          <cell r="E33">
+            <v>130000</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8">
+        <row r="5">
+          <cell r="C5" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D5" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E5" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G5" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H5">
+            <v>50000</v>
+          </cell>
+          <cell r="J5">
+            <v>1</v>
+          </cell>
+          <cell r="M5">
+            <v>0</v>
+          </cell>
+          <cell r="O5">
+            <v>0</v>
+          </cell>
+          <cell r="R5" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="C6" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D6" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E6" t="str">
+            <v>Self-employed</v>
+          </cell>
+          <cell r="G6" t="str">
+            <v>2025-08</v>
+          </cell>
+          <cell r="H6">
+            <v>70000</v>
+          </cell>
+          <cell r="J6">
+            <v>1</v>
+          </cell>
+          <cell r="M6">
+            <v>0</v>
+          </cell>
+          <cell r="O6">
+            <v>8.5487172896137054E-11</v>
+          </cell>
+          <cell r="R6" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="C7" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D7" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E7" t="str">
+            <v>Business Owner</v>
+          </cell>
+          <cell r="G7" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H7">
+            <v>90000</v>
+          </cell>
+          <cell r="J7">
+            <v>1</v>
+          </cell>
+          <cell r="M7">
+            <v>61000.000000000102</v>
+          </cell>
+          <cell r="O7">
+            <v>57607.003891050575</v>
+          </cell>
+          <cell r="R7" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="C8" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D8" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E8" t="str">
+            <v>Salaried</v>
+          </cell>
+          <cell r="G8" t="str">
+            <v>2025-09</v>
+          </cell>
+          <cell r="H8">
+            <v>110000</v>
+          </cell>
+          <cell r="J8">
+            <v>1</v>
+          </cell>
+          <cell r="M8">
+            <v>126200.0000000001</v>
+          </cell>
+          <cell r="O8">
+            <v>110000</v>
+          </cell>
+          <cell r="R8" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="C9" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D9" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E9" t="str">
+            <v>Freelancer</v>
+          </cell>
+          <cell r="G9" t="str">
+            <v>2025-10</v>
+          </cell>
+          <cell r="H9">
+            <v>130000</v>
+          </cell>
+          <cell r="J9">
+            <v>1</v>
+          </cell>
+          <cell r="M9">
+            <v>0</v>
+          </cell>
+          <cell r="O9">
+            <v>1.0103029524088925E-10</v>
+          </cell>
+          <cell r="R9" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="C10" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D10" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E10" t="str">
+            <v>Business Owner</v>
+          </cell>
+          <cell r="G10" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H10">
+            <v>150000</v>
+          </cell>
+          <cell r="J10">
+            <v>1</v>
+          </cell>
+          <cell r="M10">
+            <v>4.0745362639427185E-10</v>
+          </cell>
+          <cell r="O10">
+            <v>2.4980018054066022E-10</v>
+          </cell>
+          <cell r="R10" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="C11" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D11" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E11" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G11" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H11">
+            <v>170000</v>
+          </cell>
+          <cell r="J11">
+            <v>1</v>
+          </cell>
+          <cell r="M11">
+            <v>0</v>
+          </cell>
+          <cell r="O11">
+            <v>0</v>
+          </cell>
+          <cell r="R11" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="C12" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D12" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E12" t="str">
+            <v>Contractor</v>
+          </cell>
+          <cell r="G12" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H12">
+            <v>60000</v>
+          </cell>
+          <cell r="J12">
+            <v>1</v>
+          </cell>
+          <cell r="M12">
+            <v>0</v>
+          </cell>
+          <cell r="O12">
+            <v>8.659739592076221E-11</v>
+          </cell>
+          <cell r="R12" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="C13" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D13" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E13" t="str">
+            <v>Self-employed</v>
+          </cell>
+          <cell r="G13" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H13">
+            <v>80000</v>
+          </cell>
+          <cell r="J13">
+            <v>1</v>
+          </cell>
+          <cell r="M13">
+            <v>49066.666666666599</v>
+          </cell>
+          <cell r="O13">
+            <v>42852.983988355205</v>
+          </cell>
+          <cell r="R13" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="C14" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D14" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E14" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G14" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H14">
+            <v>100000</v>
+          </cell>
+          <cell r="J14">
+            <v>1</v>
+          </cell>
+          <cell r="M14">
+            <v>114999.9999999999</v>
+          </cell>
+          <cell r="O14">
+            <v>100000</v>
+          </cell>
+          <cell r="R14" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D15" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E15" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G15" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H15">
+            <v>120000</v>
+          </cell>
+          <cell r="J15">
+            <v>1</v>
+          </cell>
+          <cell r="M15">
+            <v>0</v>
+          </cell>
+          <cell r="O15">
+            <v>0</v>
+          </cell>
+          <cell r="R15" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D16" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E16" t="str">
+            <v>Self-employed</v>
+          </cell>
+          <cell r="G16" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H16">
+            <v>140000</v>
+          </cell>
+          <cell r="J16">
+            <v>1</v>
+          </cell>
+          <cell r="M16">
+            <v>4.0745362639427185E-10</v>
+          </cell>
+          <cell r="O16">
+            <v>2.4868995751603507E-10</v>
+          </cell>
+          <cell r="R16" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="C17" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D17" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E17" t="str">
+            <v>Business Owner</v>
+          </cell>
+          <cell r="G17" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H17">
+            <v>160000</v>
+          </cell>
+          <cell r="J17">
+            <v>1</v>
+          </cell>
+          <cell r="M17">
+            <v>0</v>
+          </cell>
+          <cell r="O17">
+            <v>0</v>
+          </cell>
+          <cell r="R17" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="C18" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D18" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E18" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G18" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H18">
+            <v>180000</v>
+          </cell>
+          <cell r="J18">
+            <v>1</v>
+          </cell>
+          <cell r="M18">
+            <v>0</v>
+          </cell>
+          <cell r="O18">
+            <v>0</v>
+          </cell>
+          <cell r="R18" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="C19" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D19" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E19" t="str">
+            <v>Freelancer</v>
+          </cell>
+          <cell r="G19" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H19">
+            <v>200000</v>
+          </cell>
+          <cell r="J19">
+            <v>1</v>
+          </cell>
+          <cell r="M19">
+            <v>228999.99999999988</v>
+          </cell>
+          <cell r="O19">
+            <v>200000</v>
+          </cell>
+          <cell r="R19" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="C20" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D20" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E20" t="str">
+            <v>Business Owner</v>
+          </cell>
+          <cell r="G20" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H20">
+            <v>70000</v>
+          </cell>
+          <cell r="J20">
+            <v>1</v>
+          </cell>
+          <cell r="M20">
+            <v>80400</v>
+          </cell>
+          <cell r="O20">
+            <v>70000</v>
+          </cell>
+          <cell r="R20" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="C21" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D21" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E21" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G21" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H21">
+            <v>90000</v>
+          </cell>
+          <cell r="J21">
+            <v>1</v>
+          </cell>
+          <cell r="M21">
+            <v>0</v>
+          </cell>
+          <cell r="O21">
+            <v>0</v>
+          </cell>
+          <cell r="R21" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="C22" t="str">
+            <v>Business Loan</v>
+          </cell>
+          <cell r="D22" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E22" t="str">
+            <v>Contractor</v>
+          </cell>
+          <cell r="G22" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H22">
+            <v>110000</v>
+          </cell>
+          <cell r="J22">
+            <v>1</v>
+          </cell>
+          <cell r="M22">
+            <v>126200.0000000001</v>
+          </cell>
+          <cell r="O22">
+            <v>110000</v>
+          </cell>
+          <cell r="R22" t="str">
+            <v>90+</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="C23" t="str">
+            <v>Salary Advance</v>
+          </cell>
+          <cell r="D23" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E23" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G23" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H23">
+            <v>50000</v>
+          </cell>
+          <cell r="J23">
+            <v>1</v>
+          </cell>
+          <cell r="M23">
+            <v>0</v>
+          </cell>
+          <cell r="O23">
+            <v>0</v>
+          </cell>
+          <cell r="R23" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="C24" t="str">
+            <v>Personal Loan</v>
+          </cell>
+          <cell r="D24" t="str">
+            <v>Unknown</v>
+          </cell>
+          <cell r="E24" t="str">
+            <v>Employee</v>
+          </cell>
+          <cell r="G24" t="str">
+            <v>2025-07</v>
+          </cell>
+          <cell r="H24">
+            <v>75000</v>
+          </cell>
+          <cell r="J24">
+            <v>1</v>
+          </cell>
+          <cell r="M24">
+            <v>0</v>
+          </cell>
+          <cell r="O24">
+            <v>9.1593399531575415E-11</v>
+          </cell>
+          <cell r="R24" t="str">
+            <v>Current</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2029,265 +4064,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="22.1796875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="82.26953125" style="47" customWidth="1"/>
-    <col min="3" max="3" width="52.1796875" style="5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
-        <v>188</v>
-      </c>
-      <c r="B1" s="41" t="s">
-        <v>189</v>
-      </c>
-      <c r="C1" s="45" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A2" s="42" t="s">
-        <v>191</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>192</v>
-      </c>
-      <c r="C2" s="46" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A3" s="42" t="s">
-        <v>194</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="42" t="s">
-        <v>197</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>198</v>
-      </c>
-      <c r="C4" s="46" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="42" t="s">
-        <v>200</v>
-      </c>
-      <c r="B5" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A6" s="42" t="s">
-        <v>203</v>
-      </c>
-      <c r="B6" s="43" t="s">
-        <v>204</v>
-      </c>
-      <c r="C6" s="46" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A7" s="42" t="s">
-        <v>206</v>
-      </c>
-      <c r="B7" s="43" t="s">
-        <v>207</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="42" t="s">
-        <v>209</v>
-      </c>
-      <c r="B8" s="43" t="s">
-        <v>210</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="42" t="s">
-        <v>212</v>
-      </c>
-      <c r="B9" s="43" t="s">
-        <v>213</v>
-      </c>
-      <c r="C9" s="46" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A10" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="B10" s="43" t="s">
-        <v>215</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="42" t="s">
-        <v>217</v>
-      </c>
-      <c r="B11" s="43" t="s">
-        <v>218</v>
-      </c>
-      <c r="C11" s="46" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="42" t="s">
-        <v>220</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>221</v>
-      </c>
-      <c r="C12" s="46" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="42" t="s">
-        <v>223</v>
-      </c>
-      <c r="B13" s="43" t="s">
-        <v>224</v>
-      </c>
-      <c r="C13" s="46" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A14" s="42" t="s">
-        <v>226</v>
-      </c>
-      <c r="B14" s="43" t="s">
-        <v>227</v>
-      </c>
-      <c r="C14" s="46" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="42" t="s">
-        <v>229</v>
-      </c>
-      <c r="B15" s="43" t="s">
-        <v>230</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="42" t="s">
-        <v>232</v>
-      </c>
-      <c r="B16" s="43" t="s">
-        <v>233</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="42" t="s">
-        <v>235</v>
-      </c>
-      <c r="B17" s="43" t="s">
-        <v>236</v>
-      </c>
-      <c r="C17" s="46" t="s">
-        <v>237</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7265625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.36328125" style="2" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>238</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B2" s="2">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>242</v>
-      </c>
-      <c r="B3" s="2">
-        <v>60</v>
-      </c>
-      <c r="C3" s="2">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="46" t="s">
-        <v>243</v>
-      </c>
-      <c r="B4" s="12">
-        <f>SUM(Loan!E2:E21)</f>
-        <v>2205000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3044,7 +4820,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4173,7 +5949,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4954,7 +6730,7 @@
         <v>49533.333333333336</v>
       </c>
       <c r="H15" s="12">
-        <f t="shared" ref="H15:H16" si="9">MAX(0,D15-I15)</f>
+        <f t="shared" ref="H15" si="9">MAX(0,D15-I15)</f>
         <v>0</v>
       </c>
       <c r="I15" s="12">
@@ -7335,7 +9111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7473,4 +9249,1045 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.1796875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="82.26953125" style="47" customWidth="1"/>
+    <col min="3" max="3" width="52.1796875" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="44" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="41" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1" s="45" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A2" s="42" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" s="46" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A3" s="42" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="C3" s="46" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="42" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="46" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="42" t="s">
+        <v>200</v>
+      </c>
+      <c r="B5" s="43" t="s">
+        <v>201</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A6" s="42" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" s="43" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A7" s="42" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>207</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="42" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="42" t="s">
+        <v>212</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>213</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A10" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>215</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="42" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="43" t="s">
+        <v>218</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="42" t="s">
+        <v>220</v>
+      </c>
+      <c r="B12" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="42" t="s">
+        <v>223</v>
+      </c>
+      <c r="B13" s="43" t="s">
+        <v>224</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A14" s="42" t="s">
+        <v>226</v>
+      </c>
+      <c r="B14" s="43" t="s">
+        <v>227</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="42" t="s">
+        <v>229</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>230</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="42" t="s">
+        <v>232</v>
+      </c>
+      <c r="B16" s="43" t="s">
+        <v>233</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="38.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="42" t="s">
+        <v>235</v>
+      </c>
+      <c r="B17" s="43" t="s">
+        <v>236</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>237</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="33.36328125" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="2">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3" s="2">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A4" s="46" t="s">
+        <v>243</v>
+      </c>
+      <c r="B4" s="12">
+        <f>SUM(Loan!E2:E21)</f>
+        <v>2205000</v>
+      </c>
+      <c r="C4" s="18">
+        <f>B4</f>
+        <v>2205000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A5" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="C5" s="12">
+        <f>SUM(Loan!J2:J21)</f>
+        <v>2520300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="26" x14ac:dyDescent="0.35">
+      <c r="A6" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="C6" s="12">
+        <f>SUM(Installment!I33:I61)</f>
+        <v>2637400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:U46"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="3" style="48" customWidth="1"/>
+    <col min="2" max="15" width="15" style="48" customWidth="1"/>
+    <col min="16" max="16" width="10" style="48" customWidth="1"/>
+    <col min="21" max="21" width="1" style="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="U1" s="49"/>
+    </row>
+    <row r="2" spans="2:21" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="U2" s="49"/>
+    </row>
+    <row r="3" spans="2:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="51" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="52" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="53" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="54">
+        <v>46050</v>
+      </c>
+      <c r="D6" s="54"/>
+      <c r="F6" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+    </row>
+    <row r="7" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="53" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D7" s="56"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="55"/>
+      <c r="I7" s="55"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55"/>
+    </row>
+    <row r="8" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="53" t="s">
+        <v>229</v>
+      </c>
+      <c r="C8" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D8" s="56"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+    </row>
+    <row r="9" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="53" t="s">
+        <v>226</v>
+      </c>
+      <c r="C9" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D9" s="56"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+    </row>
+    <row r="11" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="52" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="51" t="str">
+        <f>"As of "&amp;TEXT($C$6,"dd mmm yyyy")&amp;"  |  Product: "&amp;$C$7&amp;"  |  Channel: "&amp;$C$8&amp;"  |  Customer Type: "&amp;$C$9</f>
+        <v>As of 28 Jan 2026  |  Product: All  |  Channel: All  |  Customer Type: All</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="57" t="s">
+        <v>194</v>
+      </c>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="57" t="s">
+        <v>197</v>
+      </c>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="57" t="s">
+        <v>200</v>
+      </c>
+      <c r="I13" s="57"/>
+      <c r="J13" s="57"/>
+      <c r="K13" s="57" t="s">
+        <v>203</v>
+      </c>
+      <c r="L13" s="57"/>
+      <c r="M13" s="57"/>
+      <c r="N13" s="57" t="s">
+        <v>206</v>
+      </c>
+      <c r="O13" s="57"/>
+      <c r="P13" s="57"/>
+      <c r="Q13" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="R13" s="57"/>
+      <c r="S13" s="57"/>
+    </row>
+    <row r="14" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="58">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0))</f>
+        <v>20</v>
+      </c>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="58">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*('[1]Calc - Loan Summary'!$O$5:$O$24&gt;0)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0))</f>
+        <v>13</v>
+      </c>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59">
+        <f>SUM(Installment!H8:H61)</f>
+        <v>431666.66666666657</v>
+      </c>
+      <c r="I14" s="59"/>
+      <c r="J14" s="59"/>
+      <c r="K14" s="59">
+        <f>SUM(Installment!D2:D61)</f>
+        <v>2520299.9999999995</v>
+      </c>
+      <c r="L14" s="59"/>
+      <c r="M14" s="59"/>
+      <c r="N14" s="59">
+        <f>SUM(Installment!J2:J61)</f>
+        <v>3416466.666666667</v>
+      </c>
+      <c r="O14" s="59"/>
+      <c r="P14" s="59"/>
+      <c r="Q14" s="60">
+        <f>IFERROR(N14/K14,0)</f>
+        <v>1.3555793622452357</v>
+      </c>
+      <c r="R14" s="60"/>
+      <c r="S14" s="60"/>
+    </row>
+    <row r="15" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="58"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="59"/>
+      <c r="J15" s="59"/>
+      <c r="K15" s="59"/>
+      <c r="L15" s="59"/>
+      <c r="M15" s="59"/>
+      <c r="N15" s="59"/>
+      <c r="O15" s="59"/>
+      <c r="P15" s="59"/>
+      <c r="Q15" s="60"/>
+      <c r="R15" s="60"/>
+      <c r="S15" s="60"/>
+    </row>
+    <row r="16" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="58"/>
+      <c r="C16" s="58"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58"/>
+      <c r="H16" s="59"/>
+      <c r="I16" s="59"/>
+      <c r="J16" s="59"/>
+      <c r="K16" s="59"/>
+      <c r="L16" s="59"/>
+      <c r="M16" s="59"/>
+      <c r="N16" s="59"/>
+      <c r="O16" s="59"/>
+      <c r="P16" s="59"/>
+      <c r="Q16" s="60"/>
+      <c r="R16" s="60"/>
+      <c r="S16" s="60"/>
+    </row>
+    <row r="18" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="52" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="61" t="s">
+        <v>220</v>
+      </c>
+      <c r="C19" s="61" t="s">
+        <v>253</v>
+      </c>
+      <c r="D19" s="61" t="s">
+        <v>254</v>
+      </c>
+      <c r="E19" s="61" t="s">
+        <v>255</v>
+      </c>
+      <c r="F19" s="61" t="s">
+        <v>256</v>
+      </c>
+      <c r="G19" s="61" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="62" t="s">
+        <v>258</v>
+      </c>
+      <c r="C20" s="63">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20))</f>
+        <v>11</v>
+      </c>
+      <c r="D20" s="64">
+        <f>IFERROR(C20/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E20" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
+        <v>3.6470826358936392E-10</v>
+      </c>
+      <c r="G20" s="64">
+        <f>IFERROR(F20/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>5.2821056975290308E-16</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="62" t="s">
+        <v>259</v>
+      </c>
+      <c r="C21" s="63">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21))</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="64">
+        <f>IFERROR(C21/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="64">
+        <f>IFERROR(F21/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="62" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22" s="63">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22))</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="64">
+        <f>IFERROR(C22/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="64">
+        <f>IFERROR(F22/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="62" t="s">
+        <v>261</v>
+      </c>
+      <c r="C23" s="63">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23))</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="64">
+        <f>IFERROR(C23/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="64">
+        <f>IFERROR(F23/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="66" t="s">
+        <v>262</v>
+      </c>
+      <c r="C24" s="67">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24))</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="68">
+        <f>IFERROR(C24/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="69">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="69">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="68">
+        <f>IFERROR(F24/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="66" t="s">
+        <v>263</v>
+      </c>
+      <c r="C25" s="67">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B25))</f>
+        <v>9</v>
+      </c>
+      <c r="D25" s="68">
+        <f>IFERROR(C25/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
+        <v>0.45</v>
+      </c>
+      <c r="E25" s="69">
+        <f>SUM(Installment!K4:K61)</f>
+        <v>734866.66666666663</v>
+      </c>
+      <c r="F25" s="69">
+        <f>SUM(Table1[outstanding])</f>
+        <v>431666.66666666657</v>
+      </c>
+      <c r="G25" s="68">
+        <f>IFERROR(F25/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
+        <v>0.62518708432683279</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="70" t="s">
+        <v>264</v>
+      </c>
+      <c r="C26" s="70">
+        <f>SUM(C20:C25)</f>
+        <v>20</v>
+      </c>
+      <c r="D26" s="71">
+        <f>SUM(D20:D25)</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="72">
+        <f>SUM(E20:E25)</f>
+        <v>734866.66666666663</v>
+      </c>
+      <c r="F26" s="72">
+        <f>SUM(F20:F25)</f>
+        <v>431666.66666666692</v>
+      </c>
+      <c r="G26" s="71">
+        <f>SUM(G20:G25)</f>
+        <v>0.62518708432683334</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="52" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="61" t="s">
+        <v>223</v>
+      </c>
+      <c r="C29" s="61" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="61" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="61" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="62" t="s">
+        <v>266</v>
+      </c>
+      <c r="C30" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>530000</v>
+      </c>
+      <c r="D30" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>935000</v>
+      </c>
+      <c r="E30" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>430000</v>
+      </c>
+      <c r="F30" s="73">
+        <f>SUM(C30:E30)</f>
+        <v>1895000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="62" t="s">
+        <v>267</v>
+      </c>
+      <c r="C31" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>70000</v>
+      </c>
+      <c r="F31" s="73">
+        <f>SUM(C31:E31)</f>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="62" t="s">
+        <v>268</v>
+      </c>
+      <c r="C32" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>110000</v>
+      </c>
+      <c r="D32" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="73">
+        <f>SUM(C32:E32)</f>
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="33" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="62" t="s">
+        <v>269</v>
+      </c>
+      <c r="C33" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="65">
+        <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
+        <v>130000</v>
+      </c>
+      <c r="F33" s="73">
+        <f>SUM(C33:E33)</f>
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="34" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="70" t="s">
+        <v>264</v>
+      </c>
+      <c r="C34" s="72">
+        <f>SUM(C30:C33)</f>
+        <v>640000</v>
+      </c>
+      <c r="D34" s="72">
+        <f>SUM(D30:D33)</f>
+        <v>935000</v>
+      </c>
+      <c r="E34" s="72">
+        <f>SUM(E30:E33)</f>
+        <v>630000</v>
+      </c>
+      <c r="F34" s="72">
+        <f>SUM(F30:F33)</f>
+        <v>2205000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="74" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="52" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="75" t="s">
+        <v>272</v>
+      </c>
+      <c r="C38" s="75"/>
+      <c r="D38" s="75"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
+      <c r="H38" s="75"/>
+      <c r="I38" s="75"/>
+      <c r="J38" s="75"/>
+      <c r="K38" s="75"/>
+      <c r="L38" s="75"/>
+      <c r="M38" s="75"/>
+      <c r="N38" s="75"/>
+      <c r="O38" s="75"/>
+    </row>
+    <row r="39" spans="2:15" ht="84.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="76" t="s">
+        <v>273</v>
+      </c>
+      <c r="C39" s="76"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
+      <c r="I39" s="76"/>
+      <c r="J39" s="76"/>
+      <c r="K39" s="76"/>
+      <c r="L39" s="76"/>
+      <c r="M39" s="76"/>
+      <c r="N39" s="76"/>
+      <c r="O39" s="76"/>
+    </row>
+    <row r="40" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B40" s="77" t="s">
+        <v>274</v>
+      </c>
+      <c r="C40" s="76" t="s">
+        <v>275</v>
+      </c>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
+      <c r="I40" s="76"/>
+      <c r="J40" s="76"/>
+      <c r="K40" s="76"/>
+      <c r="L40" s="76"/>
+      <c r="M40" s="76"/>
+      <c r="N40" s="76"/>
+      <c r="O40" s="76"/>
+    </row>
+    <row r="41" spans="2:15" ht="64.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B41" s="78" t="s">
+        <v>276</v>
+      </c>
+      <c r="C41" s="76" t="s">
+        <v>277</v>
+      </c>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
+      <c r="I41" s="76"/>
+      <c r="J41" s="76"/>
+      <c r="K41" s="76"/>
+      <c r="L41" s="76"/>
+      <c r="M41" s="76"/>
+      <c r="N41" s="76"/>
+      <c r="O41" s="76"/>
+    </row>
+    <row r="42" spans="2:15" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="79"/>
+    </row>
+    <row r="43" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B43" s="75" t="s">
+        <v>278</v>
+      </c>
+      <c r="C43" s="75"/>
+      <c r="D43" s="75"/>
+      <c r="E43" s="75"/>
+      <c r="F43" s="75"/>
+      <c r="G43" s="75"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="75"/>
+      <c r="J43" s="75"/>
+      <c r="K43" s="75"/>
+      <c r="L43" s="75"/>
+      <c r="M43" s="75"/>
+      <c r="N43" s="75"/>
+      <c r="O43" s="75"/>
+    </row>
+    <row r="44" spans="2:15" ht="69.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B44" s="76" t="s">
+        <v>279</v>
+      </c>
+      <c r="C44" s="76"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
+      <c r="I44" s="76"/>
+      <c r="J44" s="76"/>
+      <c r="K44" s="76"/>
+      <c r="L44" s="76"/>
+      <c r="M44" s="76"/>
+      <c r="N44" s="76"/>
+      <c r="O44" s="76"/>
+    </row>
+    <row r="45" spans="2:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B45" s="77" t="s">
+        <v>274</v>
+      </c>
+      <c r="C45" s="76" t="s">
+        <v>280</v>
+      </c>
+      <c r="D45" s="76"/>
+      <c r="E45" s="76"/>
+      <c r="F45" s="76"/>
+      <c r="G45" s="76"/>
+      <c r="H45" s="76"/>
+      <c r="I45" s="76"/>
+      <c r="J45" s="76"/>
+      <c r="K45" s="76"/>
+      <c r="L45" s="76"/>
+      <c r="M45" s="76"/>
+      <c r="N45" s="76"/>
+      <c r="O45" s="76"/>
+    </row>
+    <row r="46" spans="2:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="77" t="s">
+        <v>276</v>
+      </c>
+      <c r="C46" s="76" t="s">
+        <v>281</v>
+      </c>
+      <c r="D46" s="76"/>
+      <c r="E46" s="76"/>
+      <c r="F46" s="76"/>
+      <c r="G46" s="76"/>
+      <c r="H46" s="76"/>
+      <c r="I46" s="76"/>
+      <c r="J46" s="76"/>
+      <c r="K46" s="76"/>
+      <c r="L46" s="76"/>
+      <c r="M46" s="76"/>
+      <c r="N46" s="76"/>
+      <c r="O46" s="76"/>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="C45:O45"/>
+    <mergeCell ref="C46:O46"/>
+    <mergeCell ref="B38:O38"/>
+    <mergeCell ref="B39:O39"/>
+    <mergeCell ref="C40:O40"/>
+    <mergeCell ref="C41:O41"/>
+    <mergeCell ref="B43:O43"/>
+    <mergeCell ref="B44:O44"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="Q13:S13"/>
+    <mergeCell ref="B14:D16"/>
+    <mergeCell ref="E14:G16"/>
+    <mergeCell ref="H14:J16"/>
+    <mergeCell ref="K14:M16"/>
+    <mergeCell ref="N14:P16"/>
+    <mergeCell ref="Q14:S16"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="F6:L9"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="K13:M13"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="list" sqref="C9">
+      <formula1>"All,Business Owner,Contractor,Employee,Freelancer,Salaried,Self-employed"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" sqref="C8">
+      <formula1>"All,Unknown"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" sqref="C7">
+      <formula1>"All,Business Loan,Personal Loan,Salary Advance"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="date" showErrorMessage="1" errorTitle="Invalid date" error="Enter a date between 2025-07-01 and 2027-12-31." sqref="C6">
+      <formula1>DATE(2025,7,1)</formula1>
+      <formula2>DATE(2027,12,31)</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Synthetic Data for Week 1 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="4" r:id="rId1"/>
@@ -889,9 +889,9 @@
   <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="167" formatCode="\₦#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="\₦#,##0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -1197,23 +1197,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="14" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1221,25 +1204,19 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="167" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="166" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -1247,6 +1224,29 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1414,7 +1414,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1556,11 +1555,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="356125320"/>
-        <c:axId val="356125712"/>
+        <c:axId val="11162648"/>
+        <c:axId val="11165392"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="356125320"/>
+        <c:axId val="11162648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1592,7 +1591,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1627,7 +1625,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="356125712"/>
+        <c:crossAx val="11165392"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1635,7 +1633,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="356125712"/>
+        <c:axId val="11165392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1676,7 +1674,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1711,7 +1708,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="356125320"/>
+        <c:crossAx val="11162648"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1785,7 +1782,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2126,11 +2122,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="356127280"/>
-        <c:axId val="356128848"/>
+        <c:axId val="11160296"/>
+        <c:axId val="11158336"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="356127280"/>
+        <c:axId val="11160296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2162,7 +2158,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2197,7 +2192,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="356128848"/>
+        <c:crossAx val="11158336"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2205,7 +2200,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="356128848"/>
+        <c:axId val="11158336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2246,7 +2241,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2281,7 +2275,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="356127280"/>
+        <c:crossAx val="11160296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2294,7 +2288,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -9566,67 +9559,67 @@
       <c r="B6" s="53" t="s">
         <v>191</v>
       </c>
-      <c r="C6" s="54">
+      <c r="C6" s="77">
         <v>46050</v>
       </c>
-      <c r="D6" s="54"/>
-      <c r="F6" s="55" t="s">
+      <c r="D6" s="77"/>
+      <c r="F6" s="78" t="s">
         <v>249</v>
       </c>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="55"/>
-      <c r="J6" s="55"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="55"/>
+      <c r="G6" s="78"/>
+      <c r="H6" s="78"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="78"/>
+      <c r="K6" s="78"/>
+      <c r="L6" s="78"/>
     </row>
     <row r="7" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="53" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="79" t="s">
         <v>250</v>
       </c>
-      <c r="D7" s="56"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
+      <c r="D7" s="79"/>
+      <c r="F7" s="78"/>
+      <c r="G7" s="78"/>
+      <c r="H7" s="78"/>
+      <c r="I7" s="78"/>
+      <c r="J7" s="78"/>
+      <c r="K7" s="78"/>
+      <c r="L7" s="78"/>
     </row>
     <row r="8" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="53" t="s">
         <v>229</v>
       </c>
-      <c r="C8" s="56" t="s">
+      <c r="C8" s="79" t="s">
         <v>250</v>
       </c>
-      <c r="D8" s="56"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="55"/>
+      <c r="D8" s="79"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="78"/>
+      <c r="L8" s="78"/>
     </row>
     <row r="9" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="53" t="s">
         <v>226</v>
       </c>
-      <c r="C9" s="56" t="s">
+      <c r="C9" s="79" t="s">
         <v>250</v>
       </c>
-      <c r="D9" s="56"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="55"/>
-      <c r="L9" s="55"/>
+      <c r="D9" s="79"/>
+      <c r="F9" s="78"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="78"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="78"/>
     </row>
     <row r="11" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="52" t="s">
@@ -9640,114 +9633,114 @@
       </c>
     </row>
     <row r="13" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="73" t="s">
         <v>194</v>
       </c>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="57" t="s">
+      <c r="C13" s="73"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="F13" s="57"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="57" t="s">
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="73" t="s">
         <v>200</v>
       </c>
-      <c r="I13" s="57"/>
-      <c r="J13" s="57"/>
-      <c r="K13" s="57" t="s">
+      <c r="I13" s="73"/>
+      <c r="J13" s="73"/>
+      <c r="K13" s="73" t="s">
         <v>203</v>
       </c>
-      <c r="L13" s="57"/>
-      <c r="M13" s="57"/>
-      <c r="N13" s="57" t="s">
+      <c r="L13" s="73"/>
+      <c r="M13" s="73"/>
+      <c r="N13" s="73" t="s">
         <v>206</v>
       </c>
-      <c r="O13" s="57"/>
-      <c r="P13" s="57"/>
-      <c r="Q13" s="57" t="s">
+      <c r="O13" s="73"/>
+      <c r="P13" s="73"/>
+      <c r="Q13" s="73" t="s">
         <v>209</v>
       </c>
-      <c r="R13" s="57"/>
-      <c r="S13" s="57"/>
+      <c r="R13" s="73"/>
+      <c r="S13" s="73"/>
     </row>
     <row r="14" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="58">
+      <c r="B14" s="74">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0))</f>
         <v>20</v>
       </c>
-      <c r="C14" s="58"/>
-      <c r="D14" s="58"/>
-      <c r="E14" s="58">
+      <c r="C14" s="74"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="74">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*('[1]Calc - Loan Summary'!$O$5:$O$24&gt;0)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0))</f>
         <v>13</v>
       </c>
-      <c r="F14" s="58"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="59">
+      <c r="F14" s="74"/>
+      <c r="G14" s="74"/>
+      <c r="H14" s="75">
         <f>SUM(Installment!H8:H61)</f>
         <v>431666.66666666657</v>
       </c>
-      <c r="I14" s="59"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="59">
+      <c r="I14" s="75"/>
+      <c r="J14" s="75"/>
+      <c r="K14" s="75">
         <f>SUM(Installment!D2:D61)</f>
         <v>2520299.9999999995</v>
       </c>
-      <c r="L14" s="59"/>
-      <c r="M14" s="59"/>
-      <c r="N14" s="59">
+      <c r="L14" s="75"/>
+      <c r="M14" s="75"/>
+      <c r="N14" s="75">
         <f>SUM(Installment!J2:J61)</f>
         <v>3416466.666666667</v>
       </c>
-      <c r="O14" s="59"/>
-      <c r="P14" s="59"/>
-      <c r="Q14" s="60">
+      <c r="O14" s="75"/>
+      <c r="P14" s="75"/>
+      <c r="Q14" s="76">
         <f>IFERROR(N14/K14,0)</f>
         <v>1.3555793622452357</v>
       </c>
-      <c r="R14" s="60"/>
-      <c r="S14" s="60"/>
+      <c r="R14" s="76"/>
+      <c r="S14" s="76"/>
     </row>
     <row r="15" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="58"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
-      <c r="M15" s="59"/>
-      <c r="N15" s="59"/>
-      <c r="O15" s="59"/>
-      <c r="P15" s="59"/>
-      <c r="Q15" s="60"/>
-      <c r="R15" s="60"/>
-      <c r="S15" s="60"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="75"/>
+      <c r="I15" s="75"/>
+      <c r="J15" s="75"/>
+      <c r="K15" s="75"/>
+      <c r="L15" s="75"/>
+      <c r="M15" s="75"/>
+      <c r="N15" s="75"/>
+      <c r="O15" s="75"/>
+      <c r="P15" s="75"/>
+      <c r="Q15" s="76"/>
+      <c r="R15" s="76"/>
+      <c r="S15" s="76"/>
     </row>
     <row r="16" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
-      <c r="F16" s="58"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="59"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="59"/>
-      <c r="O16" s="59"/>
-      <c r="P16" s="59"/>
-      <c r="Q16" s="60"/>
-      <c r="R16" s="60"/>
-      <c r="S16" s="60"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="75"/>
+      <c r="I16" s="75"/>
+      <c r="J16" s="75"/>
+      <c r="K16" s="75"/>
+      <c r="L16" s="75"/>
+      <c r="M16" s="75"/>
+      <c r="N16" s="75"/>
+      <c r="O16" s="75"/>
+      <c r="P16" s="75"/>
+      <c r="Q16" s="76"/>
+      <c r="R16" s="76"/>
+      <c r="S16" s="76"/>
     </row>
     <row r="18" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="52" t="s">
@@ -9755,196 +9748,196 @@
       </c>
     </row>
     <row r="19" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="54" t="s">
         <v>220</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="54" t="s">
         <v>253</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="54" t="s">
         <v>254</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="54" t="s">
         <v>255</v>
       </c>
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="54" t="s">
         <v>256</v>
       </c>
-      <c r="G19" s="61" t="s">
+      <c r="G19" s="54" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="55" t="s">
         <v>258</v>
       </c>
-      <c r="C20" s="63">
+      <c r="C20" s="56">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20))</f>
         <v>11</v>
       </c>
-      <c r="D20" s="64">
+      <c r="D20" s="57">
         <f>IFERROR(C20/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="E20" s="65">
+      <c r="E20" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="65">
+      <c r="F20" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B20)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
         <v>3.6470826358936392E-10</v>
       </c>
-      <c r="G20" s="64">
+      <c r="G20" s="57">
         <f>IFERROR(F20/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>5.2821056975290308E-16</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="62" t="s">
+      <c r="B21" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="C21" s="63">
+      <c r="C21" s="56">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21))</f>
         <v>0</v>
       </c>
-      <c r="D21" s="64">
+      <c r="D21" s="57">
         <f>IFERROR(C21/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="65">
+      <c r="E21" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="65">
+      <c r="F21" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B21)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="64">
+      <c r="G21" s="57">
         <f>IFERROR(F21/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="55" t="s">
         <v>260</v>
       </c>
-      <c r="C22" s="63">
+      <c r="C22" s="56">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22))</f>
         <v>0</v>
       </c>
-      <c r="D22" s="64">
+      <c r="D22" s="57">
         <f>IFERROR(C22/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="65">
+      <c r="E22" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="65">
+      <c r="F22" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B22)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="64">
+      <c r="G22" s="57">
         <f>IFERROR(F22/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="62" t="s">
+      <c r="B23" s="55" t="s">
         <v>261</v>
       </c>
-      <c r="C23" s="63">
+      <c r="C23" s="56">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23))</f>
         <v>0</v>
       </c>
-      <c r="D23" s="64">
+      <c r="D23" s="57">
         <f>IFERROR(C23/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="65">
+      <c r="E23" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="65">
+      <c r="F23" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B23)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="64">
+      <c r="G23" s="57">
         <f>IFERROR(F23/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="59" t="s">
         <v>262</v>
       </c>
-      <c r="C24" s="67">
+      <c r="C24" s="60">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24))</f>
         <v>0</v>
       </c>
-      <c r="D24" s="68">
+      <c r="D24" s="61">
         <f>IFERROR(C24/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="69">
+      <c r="E24" s="62">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24)*'[1]Calc - Loan Summary'!$M$5:$M$24)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="69">
+      <c r="F24" s="62">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B24)*'[1]Calc - Loan Summary'!$O$5:$O$24)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="68">
+      <c r="G24" s="61">
         <f>IFERROR(F24/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="66" t="s">
+      <c r="B25" s="59" t="s">
         <v>263</v>
       </c>
-      <c r="C25" s="67">
+      <c r="C25" s="60">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$R$5:$R$24=$B25))</f>
         <v>9</v>
       </c>
-      <c r="D25" s="68">
+      <c r="D25" s="61">
         <f>IFERROR(C25/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)),0)</f>
         <v>0.45</v>
       </c>
-      <c r="E25" s="69">
+      <c r="E25" s="62">
         <f>SUM(Installment!K4:K61)</f>
         <v>734866.66666666663</v>
       </c>
-      <c r="F25" s="69">
+      <c r="F25" s="62">
         <f>SUM(Table1[outstanding])</f>
         <v>431666.66666666657</v>
       </c>
-      <c r="G25" s="68">
+      <c r="G25" s="61">
         <f>IFERROR(F25/SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*'[1]Calc - Loan Summary'!$O$5:$O$24),0)</f>
         <v>0.62518708432683279</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="70" t="s">
+      <c r="B26" s="63" t="s">
         <v>264</v>
       </c>
-      <c r="C26" s="70">
+      <c r="C26" s="63">
         <f>SUM(C20:C25)</f>
         <v>20</v>
       </c>
-      <c r="D26" s="71">
+      <c r="D26" s="64">
         <f>SUM(D20:D25)</f>
         <v>1</v>
       </c>
-      <c r="E26" s="72">
+      <c r="E26" s="65">
         <f>SUM(E20:E25)</f>
         <v>734866.66666666663</v>
       </c>
-      <c r="F26" s="72">
+      <c r="F26" s="65">
         <f>SUM(F20:F25)</f>
         <v>431666.66666666692</v>
       </c>
-      <c r="G26" s="71">
+      <c r="G26" s="64">
         <f>SUM(G20:G25)</f>
         <v>0.62518708432683334</v>
       </c>
@@ -9955,129 +9948,129 @@
       </c>
     </row>
     <row r="29" spans="2:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="61" t="s">
+      <c r="B29" s="54" t="s">
         <v>223</v>
       </c>
-      <c r="C29" s="61" t="s">
+      <c r="C29" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="61" t="s">
+      <c r="D29" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="E29" s="61" t="s">
+      <c r="E29" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="F29" s="61" t="s">
+      <c r="F29" s="54" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="62" t="s">
+      <c r="B30" s="55" t="s">
         <v>266</v>
       </c>
-      <c r="C30" s="65">
+      <c r="C30" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>530000</v>
       </c>
-      <c r="D30" s="65">
+      <c r="D30" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>935000</v>
       </c>
-      <c r="E30" s="65">
+      <c r="E30" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B30)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>430000</v>
       </c>
-      <c r="F30" s="73">
+      <c r="F30" s="66">
         <f>SUM(C30:E30)</f>
         <v>1895000</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="62" t="s">
+      <c r="B31" s="55" t="s">
         <v>267</v>
       </c>
-      <c r="C31" s="65">
+      <c r="C31" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="D31" s="65">
+      <c r="D31" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="65">
+      <c r="E31" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B31)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>70000</v>
       </c>
-      <c r="F31" s="73">
+      <c r="F31" s="66">
         <f>SUM(C31:E31)</f>
         <v>70000</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="62" t="s">
+      <c r="B32" s="55" t="s">
         <v>268</v>
       </c>
-      <c r="C32" s="65">
+      <c r="C32" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>110000</v>
       </c>
-      <c r="D32" s="65">
+      <c r="D32" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="65">
+      <c r="E32" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B32)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="F32" s="73">
+      <c r="F32" s="66">
         <f>SUM(C32:E32)</f>
         <v>110000</v>
       </c>
     </row>
     <row r="33" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="62" t="s">
+      <c r="B33" s="55" t="s">
         <v>269</v>
       </c>
-      <c r="C33" s="65">
+      <c r="C33" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Business Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="65">
+      <c r="D33" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Personal Loan")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="65">
+      <c r="E33" s="58">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0)*('[1]Calc - Loan Summary'!$G$5:$G$24=$B33)*('[1]Calc - Loan Summary'!$C$5:$C$24="Salary Advance")*'[1]Calc - Loan Summary'!$H$5:$H$24)</f>
         <v>130000</v>
       </c>
-      <c r="F33" s="73">
+      <c r="F33" s="66">
         <f>SUM(C33:E33)</f>
         <v>130000</v>
       </c>
     </row>
     <row r="34" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="70" t="s">
+      <c r="B34" s="63" t="s">
         <v>264</v>
       </c>
-      <c r="C34" s="72">
+      <c r="C34" s="65">
         <f>SUM(C30:C33)</f>
         <v>640000</v>
       </c>
-      <c r="D34" s="72">
+      <c r="D34" s="65">
         <f>SUM(D30:D33)</f>
         <v>935000</v>
       </c>
-      <c r="E34" s="72">
+      <c r="E34" s="65">
         <f>SUM(E30:E33)</f>
         <v>630000</v>
       </c>
-      <c r="F34" s="72">
+      <c r="F34" s="65">
         <f>SUM(F30:F33)</f>
         <v>2205000</v>
       </c>
     </row>
     <row r="35" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="74" t="s">
+      <c r="B35" s="67" t="s">
         <v>270</v>
       </c>
     </row>
@@ -10087,162 +10080,179 @@
       </c>
     </row>
     <row r="38" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="75" t="s">
+      <c r="B38" s="72" t="s">
         <v>272</v>
       </c>
-      <c r="C38" s="75"/>
-      <c r="D38" s="75"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="75"/>
-      <c r="H38" s="75"/>
-      <c r="I38" s="75"/>
-      <c r="J38" s="75"/>
-      <c r="K38" s="75"/>
-      <c r="L38" s="75"/>
-      <c r="M38" s="75"/>
-      <c r="N38" s="75"/>
-      <c r="O38" s="75"/>
+      <c r="C38" s="72"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="72"/>
+      <c r="F38" s="72"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="72"/>
+      <c r="J38" s="72"/>
+      <c r="K38" s="72"/>
+      <c r="L38" s="72"/>
+      <c r="M38" s="72"/>
+      <c r="N38" s="72"/>
+      <c r="O38" s="72"/>
     </row>
     <row r="39" spans="2:15" ht="84.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="76" t="s">
+      <c r="B39" s="71" t="s">
         <v>273</v>
       </c>
-      <c r="C39" s="76"/>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
-      <c r="I39" s="76"/>
-      <c r="J39" s="76"/>
-      <c r="K39" s="76"/>
-      <c r="L39" s="76"/>
-      <c r="M39" s="76"/>
-      <c r="N39" s="76"/>
-      <c r="O39" s="76"/>
+      <c r="C39" s="71"/>
+      <c r="D39" s="71"/>
+      <c r="E39" s="71"/>
+      <c r="F39" s="71"/>
+      <c r="G39" s="71"/>
+      <c r="H39" s="71"/>
+      <c r="I39" s="71"/>
+      <c r="J39" s="71"/>
+      <c r="K39" s="71"/>
+      <c r="L39" s="71"/>
+      <c r="M39" s="71"/>
+      <c r="N39" s="71"/>
+      <c r="O39" s="71"/>
     </row>
     <row r="40" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="77" t="s">
+      <c r="B40" s="68" t="s">
         <v>274</v>
       </c>
-      <c r="C40" s="76" t="s">
+      <c r="C40" s="71" t="s">
         <v>275</v>
       </c>
-      <c r="D40" s="76"/>
-      <c r="E40" s="76"/>
-      <c r="F40" s="76"/>
-      <c r="G40" s="76"/>
-      <c r="H40" s="76"/>
-      <c r="I40" s="76"/>
-      <c r="J40" s="76"/>
-      <c r="K40" s="76"/>
-      <c r="L40" s="76"/>
-      <c r="M40" s="76"/>
-      <c r="N40" s="76"/>
-      <c r="O40" s="76"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="71"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="71"/>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="71"/>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
+      <c r="M40" s="71"/>
+      <c r="N40" s="71"/>
+      <c r="O40" s="71"/>
     </row>
     <row r="41" spans="2:15" ht="64.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="78" t="s">
+      <c r="B41" s="69" t="s">
         <v>276</v>
       </c>
-      <c r="C41" s="76" t="s">
+      <c r="C41" s="71" t="s">
         <v>277</v>
       </c>
-      <c r="D41" s="76"/>
-      <c r="E41" s="76"/>
-      <c r="F41" s="76"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="76"/>
-      <c r="I41" s="76"/>
-      <c r="J41" s="76"/>
-      <c r="K41" s="76"/>
-      <c r="L41" s="76"/>
-      <c r="M41" s="76"/>
-      <c r="N41" s="76"/>
-      <c r="O41" s="76"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="71"/>
+      <c r="F41" s="71"/>
+      <c r="G41" s="71"/>
+      <c r="H41" s="71"/>
+      <c r="I41" s="71"/>
+      <c r="J41" s="71"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
+      <c r="M41" s="71"/>
+      <c r="N41" s="71"/>
+      <c r="O41" s="71"/>
     </row>
     <row r="42" spans="2:15" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="79"/>
+      <c r="B42" s="70"/>
     </row>
     <row r="43" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="75" t="s">
+      <c r="B43" s="72" t="s">
         <v>278</v>
       </c>
-      <c r="C43" s="75"/>
-      <c r="D43" s="75"/>
-      <c r="E43" s="75"/>
-      <c r="F43" s="75"/>
-      <c r="G43" s="75"/>
-      <c r="H43" s="75"/>
-      <c r="I43" s="75"/>
-      <c r="J43" s="75"/>
-      <c r="K43" s="75"/>
-      <c r="L43" s="75"/>
-      <c r="M43" s="75"/>
-      <c r="N43" s="75"/>
-      <c r="O43" s="75"/>
+      <c r="C43" s="72"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="72"/>
+      <c r="F43" s="72"/>
+      <c r="G43" s="72"/>
+      <c r="H43" s="72"/>
+      <c r="I43" s="72"/>
+      <c r="J43" s="72"/>
+      <c r="K43" s="72"/>
+      <c r="L43" s="72"/>
+      <c r="M43" s="72"/>
+      <c r="N43" s="72"/>
+      <c r="O43" s="72"/>
     </row>
     <row r="44" spans="2:15" ht="69.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="76" t="s">
+      <c r="B44" s="71" t="s">
         <v>279</v>
       </c>
-      <c r="C44" s="76"/>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
-      <c r="I44" s="76"/>
-      <c r="J44" s="76"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="76"/>
-      <c r="N44" s="76"/>
-      <c r="O44" s="76"/>
+      <c r="C44" s="71"/>
+      <c r="D44" s="71"/>
+      <c r="E44" s="71"/>
+      <c r="F44" s="71"/>
+      <c r="G44" s="71"/>
+      <c r="H44" s="71"/>
+      <c r="I44" s="71"/>
+      <c r="J44" s="71"/>
+      <c r="K44" s="71"/>
+      <c r="L44" s="71"/>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
+      <c r="O44" s="71"/>
     </row>
     <row r="45" spans="2:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B45" s="77" t="s">
+      <c r="B45" s="68" t="s">
         <v>274</v>
       </c>
-      <c r="C45" s="76" t="s">
+      <c r="C45" s="71" t="s">
         <v>280</v>
       </c>
-      <c r="D45" s="76"/>
-      <c r="E45" s="76"/>
-      <c r="F45" s="76"/>
-      <c r="G45" s="76"/>
-      <c r="H45" s="76"/>
-      <c r="I45" s="76"/>
-      <c r="J45" s="76"/>
-      <c r="K45" s="76"/>
-      <c r="L45" s="76"/>
-      <c r="M45" s="76"/>
-      <c r="N45" s="76"/>
-      <c r="O45" s="76"/>
+      <c r="D45" s="71"/>
+      <c r="E45" s="71"/>
+      <c r="F45" s="71"/>
+      <c r="G45" s="71"/>
+      <c r="H45" s="71"/>
+      <c r="I45" s="71"/>
+      <c r="J45" s="71"/>
+      <c r="K45" s="71"/>
+      <c r="L45" s="71"/>
+      <c r="M45" s="71"/>
+      <c r="N45" s="71"/>
+      <c r="O45" s="71"/>
     </row>
     <row r="46" spans="2:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B46" s="77" t="s">
+      <c r="B46" s="68" t="s">
         <v>276</v>
       </c>
-      <c r="C46" s="76" t="s">
+      <c r="C46" s="71" t="s">
         <v>281</v>
       </c>
-      <c r="D46" s="76"/>
-      <c r="E46" s="76"/>
-      <c r="F46" s="76"/>
-      <c r="G46" s="76"/>
-      <c r="H46" s="76"/>
-      <c r="I46" s="76"/>
-      <c r="J46" s="76"/>
-      <c r="K46" s="76"/>
-      <c r="L46" s="76"/>
-      <c r="M46" s="76"/>
-      <c r="N46" s="76"/>
-      <c r="O46" s="76"/>
+      <c r="D46" s="71"/>
+      <c r="E46" s="71"/>
+      <c r="F46" s="71"/>
+      <c r="G46" s="71"/>
+      <c r="H46" s="71"/>
+      <c r="I46" s="71"/>
+      <c r="J46" s="71"/>
+      <c r="K46" s="71"/>
+      <c r="L46" s="71"/>
+      <c r="M46" s="71"/>
+      <c r="N46" s="71"/>
+      <c r="O46" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="F6:L9"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="Q13:S13"/>
+    <mergeCell ref="B14:D16"/>
+    <mergeCell ref="E14:G16"/>
+    <mergeCell ref="H14:J16"/>
+    <mergeCell ref="K14:M16"/>
+    <mergeCell ref="N14:P16"/>
+    <mergeCell ref="Q14:S16"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="K13:M13"/>
     <mergeCell ref="C45:O45"/>
     <mergeCell ref="C46:O46"/>
     <mergeCell ref="B38:O38"/>
@@ -10251,23 +10261,6 @@
     <mergeCell ref="C41:O41"/>
     <mergeCell ref="B43:O43"/>
     <mergeCell ref="B44:O44"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="Q13:S13"/>
-    <mergeCell ref="B14:D16"/>
-    <mergeCell ref="E14:G16"/>
-    <mergeCell ref="H14:J16"/>
-    <mergeCell ref="K14:M16"/>
-    <mergeCell ref="N14:P16"/>
-    <mergeCell ref="Q14:S16"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="F6:L9"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="K13:M13"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" sqref="C9">

</xml_diff>